<commit_message>
update save .mp4 and exel log file
</commit_message>
<xml_diff>
--- a/logs/video_history.xlsx
+++ b/logs/video_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="25.25" customWidth="1" style="1" min="1" max="1"/>
@@ -1790,6 +1790,160 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-08-10 16:51:48</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Camera_6</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>video_ok\violation_787_1786355502.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-08-10 16:51:51</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Camera_6</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>video_ng\violation_800_1786355506.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-08-10 16:51:53</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Camera_6</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>video_ng\violation_808_1786355507.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-08-10 16:51:55</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Camera_1</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>video_ng\violation_814_1786355509.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-08-10 16:52:23</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Camera_1</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>video_ng\violation_818_1786355535.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-08-10 16:52:38</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Camera_1</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>video_ok\violation_820_1786355549.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-08-10 16:53:05</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Camera_1</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>video_ng\violation_822_1786355579.mp4</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
update set start full screen
</commit_message>
<xml_diff>
--- a/logs/video_history.xlsx
+++ b/logs/video_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="25.25" customWidth="1" style="1" min="1" max="1"/>
@@ -1944,6 +1944,72 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-08-11 08:13:09</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Camera_1</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>video_ok\violation_825_1786410782.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-08-11 08:24:04</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Camera_1</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>video_ng\violation_842_1786411437.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-08-11 08:25:39</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Camera_1</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>video_ng\violation_843_1786411530.mp4</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
update font show display
</commit_message>
<xml_diff>
--- a/logs/video_history.xlsx
+++ b/logs/video_history.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D125"/>
+  <dimension ref="A1:D130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="25.25" customWidth="1" style="1" min="1" max="1"/>
@@ -3176,6 +3176,116 @@
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-09-01 11:41:12</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Camera_1</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>video_ok\violation_39756_1788237665.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-09-01 11:41:37</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Camera_1</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>video_ok\violation_39759_1788237688.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-09-01 11:41:56</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Camera_1</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>video_ok\violation_39770_1788237708.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-09-01 11:42:16</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Camera_1</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>video_ok\violation_39772_1788237727.mp4</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-09-01 11:43:17</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Camera_1</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>video_ok\violation_39780_1788237788.mp4</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>